<commit_message>
UK daily ratings for 2026-04-26
</commit_message>
<xml_diff>
--- a/output/daily_ratings/uk_ratings_2026-04-26.xlsx
+++ b/output/daily_ratings/uk_ratings_2026-04-26.xlsx
@@ -11378,26 +11378,26 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>Come On Eibhlin (IRE)</t>
+          <t>Miss Lady Grace (IRE)</t>
         </is>
       </c>
       <c r="I184" t="n">
         <v>3</v>
       </c>
       <c r="J184" t="n">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="K184" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="L184" t="n">
-        <v>2.35</v>
+        <v>2.2</v>
       </c>
       <c r="M184" t="n">
         <v>86.14</v>
       </c>
       <c r="N184" t="n">
-        <v>62.1</v>
+        <v>57.9</v>
       </c>
       <c r="O184" t="inlineStr">
         <is>
@@ -11405,7 +11405,7 @@
         </is>
       </c>
       <c r="P184" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="185">
@@ -11438,17 +11438,17 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>Miss Lady Grace (IRE)</t>
+          <t>Come On Eibhlin (IRE)</t>
         </is>
       </c>
       <c r="I185" t="n">
         <v>3</v>
       </c>
       <c r="J185" t="n">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="K185" t="n">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="L185" t="n">
         <v>2.35</v>
@@ -11457,7 +11457,7 @@
         <v>86.14</v>
       </c>
       <c r="N185" t="n">
-        <v>57.4</v>
+        <v>62.1</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -11465,7 +11465,7 @@
         </is>
       </c>
       <c r="P185" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="186">
@@ -12276,17 +12276,17 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>Shavkat</t>
+          <t>Alpine Girl (IRE)</t>
         </is>
       </c>
       <c r="I199" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J199" t="n">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="K199" t="n">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="L199" t="inlineStr"/>
       <c r="M199" t="n">
@@ -12332,17 +12332,17 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>Alpine Girl (IRE)</t>
+          <t>Shavkat</t>
         </is>
       </c>
       <c r="I200" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J200" t="n">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="K200" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="L200" t="inlineStr"/>
       <c r="M200" t="n">

</xml_diff>